<commit_message>
Auto-compress session: update summary, clean workspace
</commit_message>
<xml_diff>
--- a/projects/HR/Татьяна/tasks_registry_tatyana.xlsx
+++ b/projects/HR/Татьяна/tasks_registry_tatyana.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Реестр задач" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр задач" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр задач'!$A$1:$M$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр задач'!$A$1:$M$82</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -50,7 +50,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -73,11 +73,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -88,6 +94,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -485,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.42578125" customWidth="1" style="2" min="1" max="1"/>
@@ -5259,8 +5266,73 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Высокий</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Контроль снабжения и логистики КНР</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Сквозной мониторинг сроков китайских задач в Битрикс24</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Ежедневно проверять активность и счетчики задач в группе «Китай / Снабжение» (Группа 14) по задачам Ли Юйнань, Цянь Ин, Лиень и Азата. Если задача находится без движения или комментариев более 48 часов — оставлять пинг исполнителю и сигнализировать руководителю.</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Зависание и задержка обработки запросов фабрикам КНР устранены.</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>Татьяна</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>Артём Петров</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr">
+        <is>
+          <t>Постоянно</t>
+        </is>
+      </c>
+      <c r="L82" s="4" t="inlineStr">
+        <is>
+          <t>Новая задача (Cross-Border Bridge)</t>
+        </is>
+      </c>
+      <c r="M82" s="4" t="inlineStr">
+        <is>
+          <t>Фокусная задача трансграничного контроля. Предотвращение эффекта «кейса с брендами» на международном уровне.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M78"/>
+  <autoFilter ref="A1:M82"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>